<commit_message>
Remove Zenodo URL column from results workbook
</commit_message>
<xml_diff>
--- a/sprint 10/resultados_compilados.xlsx
+++ b/sprint 10/resultados_compilados.xlsx
@@ -5719,7 +5719,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H145"/>
+  <dimension ref="A1:G145"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="45" customWidth="1" min="1" max="1"/>
@@ -5765,11 +5765,6 @@
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>url</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
           <t>relevancia</t>
         </is>
       </c>
@@ -5802,7 +5797,6 @@
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr"/>
-      <c r="H2" s="2" t="inlineStr"/>
     </row>
     <row r="3" ht="60" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
@@ -5836,7 +5830,6 @@
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr"/>
-      <c r="H3" s="2" t="inlineStr"/>
     </row>
     <row r="4" ht="60" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
@@ -5870,7 +5863,6 @@
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr"/>
-      <c r="H4" s="2" t="inlineStr"/>
     </row>
     <row r="5" ht="60" customHeight="1">
       <c r="A5" s="2" t="inlineStr">
@@ -5904,7 +5896,6 @@
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr"/>
-      <c r="H5" s="2" t="inlineStr"/>
     </row>
     <row r="6" ht="60" customHeight="1">
       <c r="A6" s="2" t="inlineStr">
@@ -5938,7 +5929,6 @@
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr"/>
-      <c r="H6" s="2" t="inlineStr"/>
     </row>
     <row r="7" ht="60" customHeight="1">
       <c r="A7" s="2" t="inlineStr">
@@ -5968,7 +5958,6 @@
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr"/>
-      <c r="H7" s="2" t="inlineStr"/>
     </row>
     <row r="8" ht="60" customHeight="1">
       <c r="A8" s="2" t="inlineStr">
@@ -5998,7 +5987,6 @@
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr"/>
-      <c r="H8" s="2" t="inlineStr"/>
     </row>
     <row r="9" ht="60" customHeight="1">
       <c r="A9" s="2" t="inlineStr">
@@ -6028,7 +6016,6 @@
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr"/>
-      <c r="H9" s="2" t="inlineStr"/>
     </row>
     <row r="10" ht="60" customHeight="1">
       <c r="A10" s="2" t="inlineStr">
@@ -6062,7 +6049,6 @@
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr"/>
-      <c r="H10" s="2" t="inlineStr"/>
     </row>
     <row r="11" ht="60" customHeight="1">
       <c r="A11" s="2" t="inlineStr">
@@ -6092,7 +6078,6 @@
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr"/>
-      <c r="H11" s="2" t="inlineStr"/>
     </row>
     <row r="12" ht="60" customHeight="1">
       <c r="A12" s="2" t="inlineStr">
@@ -6126,7 +6111,6 @@
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr"/>
-      <c r="H12" s="2" t="inlineStr"/>
     </row>
     <row r="13" ht="60" customHeight="1">
       <c r="A13" s="2" t="inlineStr">
@@ -6160,7 +6144,6 @@
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr"/>
-      <c r="H13" s="2" t="inlineStr"/>
     </row>
     <row r="14" ht="60" customHeight="1">
       <c r="A14" s="2" t="inlineStr">
@@ -6194,7 +6177,6 @@
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr"/>
-      <c r="H14" s="2" t="inlineStr"/>
     </row>
     <row r="15" ht="60" customHeight="1">
       <c r="A15" s="2" t="inlineStr">
@@ -6228,7 +6210,6 @@
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr"/>
-      <c r="H15" s="2" t="inlineStr"/>
     </row>
     <row r="16" ht="60" customHeight="1">
       <c r="A16" s="2" t="inlineStr">
@@ -6262,7 +6243,6 @@
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr"/>
-      <c r="H16" s="2" t="inlineStr"/>
     </row>
     <row r="17" ht="60" customHeight="1">
       <c r="A17" s="2" t="inlineStr">
@@ -6296,7 +6276,6 @@
         </is>
       </c>
       <c r="G17" s="2" t="inlineStr"/>
-      <c r="H17" s="2" t="inlineStr"/>
     </row>
     <row r="18" ht="60" customHeight="1">
       <c r="A18" s="2" t="inlineStr">
@@ -6326,7 +6305,6 @@
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr"/>
-      <c r="H18" s="2" t="inlineStr"/>
     </row>
     <row r="19" ht="60" customHeight="1">
       <c r="A19" s="2" t="inlineStr">
@@ -6356,7 +6334,6 @@
         </is>
       </c>
       <c r="G19" s="2" t="inlineStr"/>
-      <c r="H19" s="2" t="inlineStr"/>
     </row>
     <row r="20" ht="60" customHeight="1">
       <c r="A20" s="2" t="inlineStr">
@@ -6386,7 +6363,6 @@
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr"/>
-      <c r="H20" s="2" t="inlineStr"/>
     </row>
     <row r="21" ht="60" customHeight="1">
       <c r="A21" s="2" t="inlineStr">
@@ -6420,7 +6396,6 @@
         </is>
       </c>
       <c r="G21" s="2" t="inlineStr"/>
-      <c r="H21" s="2" t="inlineStr"/>
     </row>
     <row r="22" ht="60" customHeight="1">
       <c r="A22" s="2" t="inlineStr">
@@ -6454,7 +6429,6 @@
         </is>
       </c>
       <c r="G22" s="2" t="inlineStr"/>
-      <c r="H22" s="2" t="inlineStr"/>
     </row>
     <row r="23" ht="60" customHeight="1">
       <c r="A23" s="2" t="inlineStr">
@@ -6488,7 +6462,6 @@
         </is>
       </c>
       <c r="G23" s="2" t="inlineStr"/>
-      <c r="H23" s="2" t="inlineStr"/>
     </row>
     <row r="24" ht="60" customHeight="1">
       <c r="A24" s="2" t="inlineStr">
@@ -6522,7 +6495,6 @@
         </is>
       </c>
       <c r="G24" s="2" t="inlineStr"/>
-      <c r="H24" s="2" t="inlineStr"/>
     </row>
     <row r="25" ht="60" customHeight="1">
       <c r="A25" s="2" t="inlineStr">
@@ -6556,7 +6528,6 @@
         </is>
       </c>
       <c r="G25" s="2" t="inlineStr"/>
-      <c r="H25" s="2" t="inlineStr"/>
     </row>
     <row r="26" ht="60" customHeight="1">
       <c r="A26" s="2" t="inlineStr">
@@ -6590,7 +6561,6 @@
         </is>
       </c>
       <c r="G26" s="2" t="inlineStr"/>
-      <c r="H26" s="2" t="inlineStr"/>
     </row>
     <row r="27" ht="60" customHeight="1">
       <c r="A27" s="2" t="inlineStr">
@@ -6624,7 +6594,6 @@
         </is>
       </c>
       <c r="G27" s="2" t="inlineStr"/>
-      <c r="H27" s="2" t="inlineStr"/>
     </row>
     <row r="28" ht="60" customHeight="1">
       <c r="A28" s="2" t="inlineStr">
@@ -6658,7 +6627,6 @@
         </is>
       </c>
       <c r="G28" s="2" t="inlineStr"/>
-      <c r="H28" s="2" t="inlineStr"/>
     </row>
     <row r="29" ht="60" customHeight="1">
       <c r="A29" s="2" t="inlineStr">
@@ -6692,7 +6660,6 @@
         </is>
       </c>
       <c r="G29" s="2" t="inlineStr"/>
-      <c r="H29" s="2" t="inlineStr"/>
     </row>
     <row r="30" ht="60" customHeight="1">
       <c r="A30" s="2" t="inlineStr">
@@ -6722,7 +6689,6 @@
         </is>
       </c>
       <c r="G30" s="2" t="inlineStr"/>
-      <c r="H30" s="2" t="inlineStr"/>
     </row>
     <row r="31" ht="60" customHeight="1">
       <c r="A31" s="2" t="inlineStr">
@@ -6752,7 +6718,6 @@
         </is>
       </c>
       <c r="G31" s="2" t="inlineStr"/>
-      <c r="H31" s="2" t="inlineStr"/>
     </row>
     <row r="32" ht="60" customHeight="1">
       <c r="A32" s="2" t="inlineStr">
@@ -6782,7 +6747,6 @@
         </is>
       </c>
       <c r="G32" s="2" t="inlineStr"/>
-      <c r="H32" s="2" t="inlineStr"/>
     </row>
     <row r="33" ht="60" customHeight="1">
       <c r="A33" s="2" t="inlineStr">
@@ -6816,7 +6780,6 @@
         </is>
       </c>
       <c r="G33" s="2" t="inlineStr"/>
-      <c r="H33" s="2" t="inlineStr"/>
     </row>
     <row r="34" ht="60" customHeight="1">
       <c r="A34" s="2" t="inlineStr">
@@ -6846,7 +6809,6 @@
         </is>
       </c>
       <c r="G34" s="2" t="inlineStr"/>
-      <c r="H34" s="2" t="inlineStr"/>
     </row>
     <row r="35" ht="60" customHeight="1">
       <c r="A35" s="2" t="inlineStr">
@@ -6880,7 +6842,6 @@
         </is>
       </c>
       <c r="G35" s="2" t="inlineStr"/>
-      <c r="H35" s="2" t="inlineStr"/>
     </row>
     <row r="36" ht="60" customHeight="1">
       <c r="A36" s="2" t="inlineStr">
@@ -6914,7 +6875,6 @@
         </is>
       </c>
       <c r="G36" s="2" t="inlineStr"/>
-      <c r="H36" s="2" t="inlineStr"/>
     </row>
     <row r="37" ht="60" customHeight="1">
       <c r="A37" s="2" t="inlineStr">
@@ -6944,7 +6904,6 @@
         </is>
       </c>
       <c r="G37" s="2" t="inlineStr"/>
-      <c r="H37" s="2" t="inlineStr"/>
     </row>
     <row r="38" ht="60" customHeight="1">
       <c r="A38" s="2" t="inlineStr">
@@ -6974,7 +6933,6 @@
         </is>
       </c>
       <c r="G38" s="2" t="inlineStr"/>
-      <c r="H38" s="2" t="inlineStr"/>
     </row>
     <row r="39" ht="60" customHeight="1">
       <c r="A39" s="2" t="inlineStr">
@@ -7004,7 +6962,6 @@
         </is>
       </c>
       <c r="G39" s="2" t="inlineStr"/>
-      <c r="H39" s="2" t="inlineStr"/>
     </row>
     <row r="40" ht="60" customHeight="1">
       <c r="A40" s="2" t="inlineStr">
@@ -7038,7 +6995,6 @@
         </is>
       </c>
       <c r="G40" s="2" t="inlineStr"/>
-      <c r="H40" s="2" t="inlineStr"/>
     </row>
     <row r="41" ht="60" customHeight="1">
       <c r="A41" s="2" t="inlineStr">
@@ -7068,7 +7024,6 @@
         </is>
       </c>
       <c r="G41" s="2" t="inlineStr"/>
-      <c r="H41" s="2" t="inlineStr"/>
     </row>
     <row r="42" ht="60" customHeight="1">
       <c r="A42" s="2" t="inlineStr">
@@ -7098,7 +7053,6 @@
         </is>
       </c>
       <c r="G42" s="2" t="inlineStr"/>
-      <c r="H42" s="2" t="inlineStr"/>
     </row>
     <row r="43" ht="60" customHeight="1">
       <c r="A43" s="2" t="inlineStr">
@@ -7128,7 +7082,6 @@
         </is>
       </c>
       <c r="G43" s="2" t="inlineStr"/>
-      <c r="H43" s="2" t="inlineStr"/>
     </row>
     <row r="44" ht="60" customHeight="1">
       <c r="A44" s="2" t="inlineStr">
@@ -7162,7 +7115,6 @@
         </is>
       </c>
       <c r="G44" s="2" t="inlineStr"/>
-      <c r="H44" s="2" t="inlineStr"/>
     </row>
     <row r="45" ht="60" customHeight="1">
       <c r="A45" s="2" t="inlineStr">
@@ -7196,7 +7148,6 @@
         </is>
       </c>
       <c r="G45" s="2" t="inlineStr"/>
-      <c r="H45" s="2" t="inlineStr"/>
     </row>
     <row r="46" ht="60" customHeight="1">
       <c r="A46" s="2" t="inlineStr">
@@ -7230,7 +7181,6 @@
         </is>
       </c>
       <c r="G46" s="2" t="inlineStr"/>
-      <c r="H46" s="2" t="inlineStr"/>
     </row>
     <row r="47" ht="60" customHeight="1">
       <c r="A47" s="2" t="inlineStr">
@@ -7264,7 +7214,6 @@
         </is>
       </c>
       <c r="G47" s="2" t="inlineStr"/>
-      <c r="H47" s="2" t="inlineStr"/>
     </row>
     <row r="48" ht="60" customHeight="1">
       <c r="A48" s="2" t="inlineStr">
@@ -7294,7 +7243,6 @@
         </is>
       </c>
       <c r="G48" s="2" t="inlineStr"/>
-      <c r="H48" s="2" t="inlineStr"/>
     </row>
     <row r="49" ht="60" customHeight="1">
       <c r="A49" s="2" t="inlineStr">
@@ -7324,7 +7272,6 @@
         </is>
       </c>
       <c r="G49" s="2" t="inlineStr"/>
-      <c r="H49" s="2" t="inlineStr"/>
     </row>
     <row r="50" ht="60" customHeight="1">
       <c r="A50" s="2" t="inlineStr">
@@ -7354,7 +7301,6 @@
         </is>
       </c>
       <c r="G50" s="2" t="inlineStr"/>
-      <c r="H50" s="2" t="inlineStr"/>
     </row>
     <row r="51" ht="60" customHeight="1">
       <c r="A51" s="2" t="inlineStr">
@@ -7388,7 +7334,6 @@
         </is>
       </c>
       <c r="G51" s="2" t="inlineStr"/>
-      <c r="H51" s="2" t="inlineStr"/>
     </row>
     <row r="52" ht="60" customHeight="1">
       <c r="A52" s="2" t="inlineStr">
@@ -7422,7 +7367,6 @@
         </is>
       </c>
       <c r="G52" s="2" t="inlineStr"/>
-      <c r="H52" s="2" t="inlineStr"/>
     </row>
     <row r="53" ht="60" customHeight="1">
       <c r="A53" s="2" t="inlineStr">
@@ -7456,7 +7400,6 @@
         </is>
       </c>
       <c r="G53" s="2" t="inlineStr"/>
-      <c r="H53" s="2" t="inlineStr"/>
     </row>
     <row r="54" ht="60" customHeight="1">
       <c r="A54" s="2" t="inlineStr">
@@ -7490,7 +7433,6 @@
         </is>
       </c>
       <c r="G54" s="2" t="inlineStr"/>
-      <c r="H54" s="2" t="inlineStr"/>
     </row>
     <row r="55" ht="60" customHeight="1">
       <c r="A55" s="2" t="inlineStr">
@@ -7524,7 +7466,6 @@
         </is>
       </c>
       <c r="G55" s="2" t="inlineStr"/>
-      <c r="H55" s="2" t="inlineStr"/>
     </row>
     <row r="56" ht="60" customHeight="1">
       <c r="A56" s="2" t="inlineStr">
@@ -7554,7 +7495,6 @@
         </is>
       </c>
       <c r="G56" s="2" t="inlineStr"/>
-      <c r="H56" s="2" t="inlineStr"/>
     </row>
     <row r="57" ht="60" customHeight="1">
       <c r="A57" s="2" t="inlineStr">
@@ -7584,7 +7524,6 @@
         </is>
       </c>
       <c r="G57" s="2" t="inlineStr"/>
-      <c r="H57" s="2" t="inlineStr"/>
     </row>
     <row r="58" ht="60" customHeight="1">
       <c r="A58" s="2" t="inlineStr">
@@ -7618,7 +7557,6 @@
         </is>
       </c>
       <c r="G58" s="2" t="inlineStr"/>
-      <c r="H58" s="2" t="inlineStr"/>
     </row>
     <row r="59" ht="60" customHeight="1">
       <c r="A59" s="2" t="inlineStr">
@@ -7648,7 +7586,6 @@
         </is>
       </c>
       <c r="G59" s="2" t="inlineStr"/>
-      <c r="H59" s="2" t="inlineStr"/>
     </row>
     <row r="60" ht="60" customHeight="1">
       <c r="A60" s="2" t="inlineStr">
@@ -7682,7 +7619,6 @@
         </is>
       </c>
       <c r="G60" s="2" t="inlineStr"/>
-      <c r="H60" s="2" t="inlineStr"/>
     </row>
     <row r="61" ht="60" customHeight="1">
       <c r="A61" s="2" t="inlineStr">
@@ -7716,7 +7652,6 @@
         </is>
       </c>
       <c r="G61" s="2" t="inlineStr"/>
-      <c r="H61" s="2" t="inlineStr"/>
     </row>
     <row r="62" ht="60" customHeight="1">
       <c r="A62" s="2" t="inlineStr">
@@ -7746,7 +7681,6 @@
         </is>
       </c>
       <c r="G62" s="2" t="inlineStr"/>
-      <c r="H62" s="2" t="inlineStr"/>
     </row>
     <row r="63" ht="60" customHeight="1">
       <c r="A63" s="2" t="inlineStr">
@@ -7780,7 +7714,6 @@
         </is>
       </c>
       <c r="G63" s="2" t="inlineStr"/>
-      <c r="H63" s="2" t="inlineStr"/>
     </row>
     <row r="64" ht="60" customHeight="1">
       <c r="A64" s="2" t="inlineStr">
@@ -7814,7 +7747,6 @@
         </is>
       </c>
       <c r="G64" s="2" t="inlineStr"/>
-      <c r="H64" s="2" t="inlineStr"/>
     </row>
     <row r="65" ht="60" customHeight="1">
       <c r="A65" s="2" t="inlineStr">
@@ -7848,7 +7780,6 @@
         </is>
       </c>
       <c r="G65" s="2" t="inlineStr"/>
-      <c r="H65" s="2" t="inlineStr"/>
     </row>
     <row r="66" ht="60" customHeight="1">
       <c r="A66" s="2" t="inlineStr">
@@ -7878,7 +7809,6 @@
         </is>
       </c>
       <c r="G66" s="2" t="inlineStr"/>
-      <c r="H66" s="2" t="inlineStr"/>
     </row>
     <row r="67" ht="60" customHeight="1">
       <c r="A67" s="2" t="inlineStr">
@@ -7908,7 +7838,6 @@
         </is>
       </c>
       <c r="G67" s="2" t="inlineStr"/>
-      <c r="H67" s="2" t="inlineStr"/>
     </row>
     <row r="68" ht="60" customHeight="1">
       <c r="A68" s="2" t="inlineStr">
@@ -7942,7 +7871,6 @@
         </is>
       </c>
       <c r="G68" s="2" t="inlineStr"/>
-      <c r="H68" s="2" t="inlineStr"/>
     </row>
     <row r="69" ht="60" customHeight="1">
       <c r="A69" s="2" t="inlineStr">
@@ -7976,7 +7904,6 @@
         </is>
       </c>
       <c r="G69" s="2" t="inlineStr"/>
-      <c r="H69" s="2" t="inlineStr"/>
     </row>
     <row r="70" ht="60" customHeight="1">
       <c r="A70" s="2" t="inlineStr">
@@ -8006,7 +7933,6 @@
         </is>
       </c>
       <c r="G70" s="2" t="inlineStr"/>
-      <c r="H70" s="2" t="inlineStr"/>
     </row>
     <row r="71" ht="60" customHeight="1">
       <c r="A71" s="2" t="inlineStr">
@@ -8036,7 +7962,6 @@
         </is>
       </c>
       <c r="G71" s="2" t="inlineStr"/>
-      <c r="H71" s="2" t="inlineStr"/>
     </row>
     <row r="72" ht="60" customHeight="1">
       <c r="A72" s="2" t="inlineStr">
@@ -8070,7 +7995,6 @@
         </is>
       </c>
       <c r="G72" s="2" t="inlineStr"/>
-      <c r="H72" s="2" t="inlineStr"/>
     </row>
     <row r="73" ht="60" customHeight="1">
       <c r="A73" s="2" t="inlineStr">
@@ -8104,7 +8028,6 @@
         </is>
       </c>
       <c r="G73" s="2" t="inlineStr"/>
-      <c r="H73" s="2" t="inlineStr"/>
     </row>
     <row r="74" ht="60" customHeight="1">
       <c r="A74" s="2" t="inlineStr">
@@ -8138,7 +8061,6 @@
         </is>
       </c>
       <c r="G74" s="2" t="inlineStr"/>
-      <c r="H74" s="2" t="inlineStr"/>
     </row>
     <row r="75" ht="60" customHeight="1">
       <c r="A75" s="2" t="inlineStr">
@@ -8172,7 +8094,6 @@
         </is>
       </c>
       <c r="G75" s="2" t="inlineStr"/>
-      <c r="H75" s="2" t="inlineStr"/>
     </row>
     <row r="76" ht="60" customHeight="1">
       <c r="A76" s="2" t="inlineStr">
@@ -8206,7 +8127,6 @@
         </is>
       </c>
       <c r="G76" s="2" t="inlineStr"/>
-      <c r="H76" s="2" t="inlineStr"/>
     </row>
     <row r="77" ht="60" customHeight="1">
       <c r="A77" s="2" t="inlineStr">
@@ -8236,7 +8156,6 @@
         </is>
       </c>
       <c r="G77" s="2" t="inlineStr"/>
-      <c r="H77" s="2" t="inlineStr"/>
     </row>
     <row r="78" ht="60" customHeight="1">
       <c r="A78" s="2" t="inlineStr">
@@ -8270,7 +8189,6 @@
         </is>
       </c>
       <c r="G78" s="2" t="inlineStr"/>
-      <c r="H78" s="2" t="inlineStr"/>
     </row>
     <row r="79" ht="60" customHeight="1">
       <c r="A79" s="2" t="inlineStr">
@@ -8300,7 +8218,6 @@
         </is>
       </c>
       <c r="G79" s="2" t="inlineStr"/>
-      <c r="H79" s="2" t="inlineStr"/>
     </row>
     <row r="80" ht="60" customHeight="1">
       <c r="A80" s="2" t="inlineStr">
@@ -8330,7 +8247,6 @@
         </is>
       </c>
       <c r="G80" s="2" t="inlineStr"/>
-      <c r="H80" s="2" t="inlineStr"/>
     </row>
     <row r="81" ht="60" customHeight="1">
       <c r="A81" s="2" t="inlineStr">
@@ -8360,7 +8276,6 @@
         </is>
       </c>
       <c r="G81" s="2" t="inlineStr"/>
-      <c r="H81" s="2" t="inlineStr"/>
     </row>
     <row r="82" ht="60" customHeight="1">
       <c r="A82" s="2" t="inlineStr">
@@ -8394,7 +8309,6 @@
         </is>
       </c>
       <c r="G82" s="2" t="inlineStr"/>
-      <c r="H82" s="2" t="inlineStr"/>
     </row>
     <row r="83" ht="60" customHeight="1">
       <c r="A83" s="2" t="inlineStr">
@@ -8424,7 +8338,6 @@
         </is>
       </c>
       <c r="G83" s="2" t="inlineStr"/>
-      <c r="H83" s="2" t="inlineStr"/>
     </row>
     <row r="84" ht="60" customHeight="1">
       <c r="A84" s="2" t="inlineStr">
@@ -8458,7 +8371,6 @@
         </is>
       </c>
       <c r="G84" s="2" t="inlineStr"/>
-      <c r="H84" s="2" t="inlineStr"/>
     </row>
     <row r="85" ht="60" customHeight="1">
       <c r="A85" s="2" t="inlineStr">
@@ -8488,7 +8400,6 @@
         </is>
       </c>
       <c r="G85" s="2" t="inlineStr"/>
-      <c r="H85" s="2" t="inlineStr"/>
     </row>
     <row r="86" ht="60" customHeight="1">
       <c r="A86" s="2" t="inlineStr">
@@ -8522,7 +8433,6 @@
         </is>
       </c>
       <c r="G86" s="2" t="inlineStr"/>
-      <c r="H86" s="2" t="inlineStr"/>
     </row>
     <row r="87" ht="60" customHeight="1">
       <c r="A87" s="2" t="inlineStr">
@@ -8552,7 +8462,6 @@
         </is>
       </c>
       <c r="G87" s="2" t="inlineStr"/>
-      <c r="H87" s="2" t="inlineStr"/>
     </row>
     <row r="88" ht="60" customHeight="1">
       <c r="A88" s="2" t="inlineStr">
@@ -8582,7 +8491,6 @@
         </is>
       </c>
       <c r="G88" s="2" t="inlineStr"/>
-      <c r="H88" s="2" t="inlineStr"/>
     </row>
     <row r="89" ht="60" customHeight="1">
       <c r="A89" s="2" t="inlineStr">
@@ -8612,7 +8520,6 @@
         </is>
       </c>
       <c r="G89" s="2" t="inlineStr"/>
-      <c r="H89" s="2" t="inlineStr"/>
     </row>
     <row r="90" ht="60" customHeight="1">
       <c r="A90" s="2" t="inlineStr">
@@ -8642,7 +8549,6 @@
         </is>
       </c>
       <c r="G90" s="2" t="inlineStr"/>
-      <c r="H90" s="2" t="inlineStr"/>
     </row>
     <row r="91" ht="60" customHeight="1">
       <c r="A91" s="2" t="inlineStr">
@@ -8672,7 +8578,6 @@
         </is>
       </c>
       <c r="G91" s="2" t="inlineStr"/>
-      <c r="H91" s="2" t="inlineStr"/>
     </row>
     <row r="92" ht="60" customHeight="1">
       <c r="A92" s="2" t="inlineStr">
@@ -8706,7 +8611,6 @@
         </is>
       </c>
       <c r="G92" s="2" t="inlineStr"/>
-      <c r="H92" s="2" t="inlineStr"/>
     </row>
     <row r="93" ht="60" customHeight="1">
       <c r="A93" s="2" t="inlineStr">
@@ -8740,7 +8644,6 @@
         </is>
       </c>
       <c r="G93" s="2" t="inlineStr"/>
-      <c r="H93" s="2" t="inlineStr"/>
     </row>
     <row r="94" ht="60" customHeight="1">
       <c r="A94" s="2" t="inlineStr">
@@ -8774,7 +8677,6 @@
         </is>
       </c>
       <c r="G94" s="2" t="inlineStr"/>
-      <c r="H94" s="2" t="inlineStr"/>
     </row>
     <row r="95" ht="60" customHeight="1">
       <c r="A95" s="2" t="inlineStr">
@@ -8804,7 +8706,6 @@
         </is>
       </c>
       <c r="G95" s="2" t="inlineStr"/>
-      <c r="H95" s="2" t="inlineStr"/>
     </row>
     <row r="96" ht="60" customHeight="1">
       <c r="A96" s="2" t="inlineStr">
@@ -8838,7 +8739,6 @@
         </is>
       </c>
       <c r="G96" s="2" t="inlineStr"/>
-      <c r="H96" s="2" t="inlineStr"/>
     </row>
     <row r="97" ht="60" customHeight="1">
       <c r="A97" s="2" t="inlineStr">
@@ -8868,7 +8768,6 @@
         </is>
       </c>
       <c r="G97" s="2" t="inlineStr"/>
-      <c r="H97" s="2" t="inlineStr"/>
     </row>
     <row r="98" ht="60" customHeight="1">
       <c r="A98" s="2" t="inlineStr">
@@ -8902,7 +8801,6 @@
         </is>
       </c>
       <c r="G98" s="2" t="inlineStr"/>
-      <c r="H98" s="2" t="inlineStr"/>
     </row>
     <row r="99" ht="60" customHeight="1">
       <c r="A99" s="2" t="inlineStr">
@@ -8936,7 +8834,6 @@
         </is>
       </c>
       <c r="G99" s="2" t="inlineStr"/>
-      <c r="H99" s="2" t="inlineStr"/>
     </row>
     <row r="100" ht="60" customHeight="1">
       <c r="A100" s="2" t="inlineStr">
@@ -8966,7 +8863,6 @@
         </is>
       </c>
       <c r="G100" s="2" t="inlineStr"/>
-      <c r="H100" s="2" t="inlineStr"/>
     </row>
     <row r="101" ht="60" customHeight="1">
       <c r="A101" s="2" t="inlineStr">
@@ -8996,7 +8892,6 @@
         </is>
       </c>
       <c r="G101" s="2" t="inlineStr"/>
-      <c r="H101" s="2" t="inlineStr"/>
     </row>
     <row r="102" ht="60" customHeight="1">
       <c r="A102" s="2" t="inlineStr">
@@ -9026,7 +8921,6 @@
         </is>
       </c>
       <c r="G102" s="2" t="inlineStr"/>
-      <c r="H102" s="2" t="inlineStr"/>
     </row>
     <row r="103" ht="60" customHeight="1">
       <c r="A103" s="2" t="inlineStr">
@@ -9056,7 +8950,6 @@
         </is>
       </c>
       <c r="G103" s="2" t="inlineStr"/>
-      <c r="H103" s="2" t="inlineStr"/>
     </row>
     <row r="104" ht="60" customHeight="1">
       <c r="A104" s="2" t="inlineStr">
@@ -9090,7 +8983,6 @@
         </is>
       </c>
       <c r="G104" s="2" t="inlineStr"/>
-      <c r="H104" s="2" t="inlineStr"/>
     </row>
     <row r="105" ht="60" customHeight="1">
       <c r="A105" s="2" t="inlineStr">
@@ -9124,7 +9016,6 @@
         </is>
       </c>
       <c r="G105" s="2" t="inlineStr"/>
-      <c r="H105" s="2" t="inlineStr"/>
     </row>
     <row r="106" ht="60" customHeight="1">
       <c r="A106" s="2" t="inlineStr">
@@ -9154,7 +9045,6 @@
         </is>
       </c>
       <c r="G106" s="2" t="inlineStr"/>
-      <c r="H106" s="2" t="inlineStr"/>
     </row>
     <row r="107" ht="60" customHeight="1">
       <c r="A107" s="2" t="inlineStr">
@@ -9184,7 +9074,6 @@
         </is>
       </c>
       <c r="G107" s="2" t="inlineStr"/>
-      <c r="H107" s="2" t="inlineStr"/>
     </row>
     <row r="108" ht="60" customHeight="1">
       <c r="A108" s="2" t="inlineStr">
@@ -9218,7 +9107,6 @@
         </is>
       </c>
       <c r="G108" s="2" t="inlineStr"/>
-      <c r="H108" s="2" t="inlineStr"/>
     </row>
     <row r="109" ht="60" customHeight="1">
       <c r="A109" s="2" t="inlineStr">
@@ -9252,7 +9140,6 @@
         </is>
       </c>
       <c r="G109" s="2" t="inlineStr"/>
-      <c r="H109" s="2" t="inlineStr"/>
     </row>
     <row r="110" ht="60" customHeight="1">
       <c r="A110" s="2" t="inlineStr">
@@ -9286,7 +9173,6 @@
         </is>
       </c>
       <c r="G110" s="2" t="inlineStr"/>
-      <c r="H110" s="2" t="inlineStr"/>
     </row>
     <row r="111" ht="60" customHeight="1">
       <c r="A111" s="2" t="inlineStr">
@@ -9320,7 +9206,6 @@
         </is>
       </c>
       <c r="G111" s="2" t="inlineStr"/>
-      <c r="H111" s="2" t="inlineStr"/>
     </row>
     <row r="112" ht="60" customHeight="1">
       <c r="A112" s="2" t="inlineStr">
@@ -9350,7 +9235,6 @@
         </is>
       </c>
       <c r="G112" s="2" t="inlineStr"/>
-      <c r="H112" s="2" t="inlineStr"/>
     </row>
     <row r="113" ht="60" customHeight="1">
       <c r="A113" s="2" t="inlineStr">
@@ -9380,7 +9264,6 @@
         </is>
       </c>
       <c r="G113" s="2" t="inlineStr"/>
-      <c r="H113" s="2" t="inlineStr"/>
     </row>
     <row r="114" ht="60" customHeight="1">
       <c r="A114" s="2" t="inlineStr">
@@ -9414,7 +9297,6 @@
         </is>
       </c>
       <c r="G114" s="2" t="inlineStr"/>
-      <c r="H114" s="2" t="inlineStr"/>
     </row>
     <row r="115" ht="60" customHeight="1">
       <c r="A115" s="2" t="inlineStr">
@@ -9444,7 +9326,6 @@
         </is>
       </c>
       <c r="G115" s="2" t="inlineStr"/>
-      <c r="H115" s="2" t="inlineStr"/>
     </row>
     <row r="116" ht="60" customHeight="1">
       <c r="A116" s="2" t="inlineStr">
@@ -9478,7 +9359,6 @@
         </is>
       </c>
       <c r="G116" s="2" t="inlineStr"/>
-      <c r="H116" s="2" t="inlineStr"/>
     </row>
     <row r="117" ht="60" customHeight="1">
       <c r="A117" s="2" t="inlineStr">
@@ -9512,7 +9392,6 @@
         </is>
       </c>
       <c r="G117" s="2" t="inlineStr"/>
-      <c r="H117" s="2" t="inlineStr"/>
     </row>
     <row r="118" ht="60" customHeight="1">
       <c r="A118" s="2" t="inlineStr">
@@ -9542,7 +9421,6 @@
         </is>
       </c>
       <c r="G118" s="2" t="inlineStr"/>
-      <c r="H118" s="2" t="inlineStr"/>
     </row>
     <row r="119" ht="60" customHeight="1">
       <c r="A119" s="2" t="inlineStr">
@@ -9576,7 +9454,6 @@
         </is>
       </c>
       <c r="G119" s="2" t="inlineStr"/>
-      <c r="H119" s="2" t="inlineStr"/>
     </row>
     <row r="120" ht="60" customHeight="1">
       <c r="A120" s="2" t="inlineStr">
@@ -9606,7 +9483,6 @@
         </is>
       </c>
       <c r="G120" s="2" t="inlineStr"/>
-      <c r="H120" s="2" t="inlineStr"/>
     </row>
     <row r="121" ht="60" customHeight="1">
       <c r="A121" s="2" t="inlineStr">
@@ -9636,7 +9512,6 @@
         </is>
       </c>
       <c r="G121" s="2" t="inlineStr"/>
-      <c r="H121" s="2" t="inlineStr"/>
     </row>
     <row r="122" ht="60" customHeight="1">
       <c r="A122" s="2" t="inlineStr">
@@ -9670,7 +9545,6 @@
         </is>
       </c>
       <c r="G122" s="2" t="inlineStr"/>
-      <c r="H122" s="2" t="inlineStr"/>
     </row>
     <row r="123" ht="60" customHeight="1">
       <c r="A123" s="2" t="inlineStr">
@@ -9704,7 +9578,6 @@
         </is>
       </c>
       <c r="G123" s="2" t="inlineStr"/>
-      <c r="H123" s="2" t="inlineStr"/>
     </row>
     <row r="124" ht="60" customHeight="1">
       <c r="A124" s="2" t="inlineStr">
@@ -9734,7 +9607,6 @@
         </is>
       </c>
       <c r="G124" s="2" t="inlineStr"/>
-      <c r="H124" s="2" t="inlineStr"/>
     </row>
     <row r="125" ht="60" customHeight="1">
       <c r="A125" s="2" t="inlineStr">
@@ -9764,7 +9636,6 @@
         </is>
       </c>
       <c r="G125" s="2" t="inlineStr"/>
-      <c r="H125" s="2" t="inlineStr"/>
     </row>
     <row r="126" ht="60" customHeight="1">
       <c r="A126" s="2" t="inlineStr">
@@ -9798,7 +9669,6 @@
         </is>
       </c>
       <c r="G126" s="2" t="inlineStr"/>
-      <c r="H126" s="2" t="inlineStr"/>
     </row>
     <row r="127" ht="60" customHeight="1">
       <c r="A127" s="2" t="inlineStr">
@@ -9832,7 +9702,6 @@
         </is>
       </c>
       <c r="G127" s="2" t="inlineStr"/>
-      <c r="H127" s="2" t="inlineStr"/>
     </row>
     <row r="128" ht="60" customHeight="1">
       <c r="A128" s="2" t="inlineStr">
@@ -9866,7 +9735,6 @@
         </is>
       </c>
       <c r="G128" s="2" t="inlineStr"/>
-      <c r="H128" s="2" t="inlineStr"/>
     </row>
     <row r="129" ht="60" customHeight="1">
       <c r="A129" s="2" t="inlineStr">
@@ -9896,7 +9764,6 @@
         </is>
       </c>
       <c r="G129" s="2" t="inlineStr"/>
-      <c r="H129" s="2" t="inlineStr"/>
     </row>
     <row r="130" ht="60" customHeight="1">
       <c r="A130" s="2" t="inlineStr">
@@ -9926,7 +9793,6 @@
         </is>
       </c>
       <c r="G130" s="2" t="inlineStr"/>
-      <c r="H130" s="2" t="inlineStr"/>
     </row>
     <row r="131" ht="60" customHeight="1">
       <c r="A131" s="2" t="inlineStr">
@@ -9960,7 +9826,6 @@
         </is>
       </c>
       <c r="G131" s="2" t="inlineStr"/>
-      <c r="H131" s="2" t="inlineStr"/>
     </row>
     <row r="132" ht="60" customHeight="1">
       <c r="A132" s="2" t="inlineStr">
@@ -9994,7 +9859,6 @@
         </is>
       </c>
       <c r="G132" s="2" t="inlineStr"/>
-      <c r="H132" s="2" t="inlineStr"/>
     </row>
     <row r="133" ht="60" customHeight="1">
       <c r="A133" s="2" t="inlineStr">
@@ -10024,7 +9888,6 @@
         </is>
       </c>
       <c r="G133" s="2" t="inlineStr"/>
-      <c r="H133" s="2" t="inlineStr"/>
     </row>
     <row r="134" ht="60" customHeight="1">
       <c r="A134" s="2" t="inlineStr">
@@ -10058,7 +9921,6 @@
         </is>
       </c>
       <c r="G134" s="2" t="inlineStr"/>
-      <c r="H134" s="2" t="inlineStr"/>
     </row>
     <row r="135" ht="60" customHeight="1">
       <c r="A135" s="2" t="inlineStr">
@@ -10088,7 +9950,6 @@
         </is>
       </c>
       <c r="G135" s="2" t="inlineStr"/>
-      <c r="H135" s="2" t="inlineStr"/>
     </row>
     <row r="136" ht="60" customHeight="1">
       <c r="A136" s="2" t="inlineStr">
@@ -10122,7 +9983,6 @@
         </is>
       </c>
       <c r="G136" s="2" t="inlineStr"/>
-      <c r="H136" s="2" t="inlineStr"/>
     </row>
     <row r="137" ht="60" customHeight="1">
       <c r="A137" s="2" t="inlineStr">
@@ -10156,7 +10016,6 @@
         </is>
       </c>
       <c r="G137" s="2" t="inlineStr"/>
-      <c r="H137" s="2" t="inlineStr"/>
     </row>
     <row r="138" ht="60" customHeight="1">
       <c r="A138" s="2" t="inlineStr">
@@ -10190,7 +10049,6 @@
         </is>
       </c>
       <c r="G138" s="2" t="inlineStr"/>
-      <c r="H138" s="2" t="inlineStr"/>
     </row>
     <row r="139" ht="60" customHeight="1">
       <c r="A139" s="2" t="inlineStr">
@@ -10224,7 +10082,6 @@
         </is>
       </c>
       <c r="G139" s="2" t="inlineStr"/>
-      <c r="H139" s="2" t="inlineStr"/>
     </row>
     <row r="140" ht="60" customHeight="1">
       <c r="A140" s="2" t="inlineStr">
@@ -10258,7 +10115,6 @@
         </is>
       </c>
       <c r="G140" s="2" t="inlineStr"/>
-      <c r="H140" s="2" t="inlineStr"/>
     </row>
     <row r="141" ht="60" customHeight="1">
       <c r="A141" s="2" t="inlineStr">
@@ -10288,7 +10144,6 @@
         </is>
       </c>
       <c r="G141" s="2" t="inlineStr"/>
-      <c r="H141" s="2" t="inlineStr"/>
     </row>
     <row r="142" ht="60" customHeight="1">
       <c r="A142" s="2" t="inlineStr">
@@ -10318,7 +10173,6 @@
         </is>
       </c>
       <c r="G142" s="2" t="inlineStr"/>
-      <c r="H142" s="2" t="inlineStr"/>
     </row>
     <row r="143" ht="60" customHeight="1">
       <c r="A143" s="2" t="inlineStr">
@@ -10348,7 +10202,6 @@
         </is>
       </c>
       <c r="G143" s="2" t="inlineStr"/>
-      <c r="H143" s="2" t="inlineStr"/>
     </row>
     <row r="144" ht="60" customHeight="1">
       <c r="A144" s="2" t="inlineStr">
@@ -10378,7 +10231,6 @@
         </is>
       </c>
       <c r="G144" s="2" t="inlineStr"/>
-      <c r="H144" s="2" t="inlineStr"/>
     </row>
     <row r="145" ht="60" customHeight="1">
       <c r="A145" s="2" t="inlineStr">
@@ -10408,7 +10260,6 @@
         </is>
       </c>
       <c r="G145" s="2" t="inlineStr"/>
-      <c r="H145" s="2" t="inlineStr"/>
     </row>
     <row r="146" ht="60" customHeight="1"/>
   </sheetData>

</xml_diff>